<commit_message>
DCC-1:2022: move per-level detail to markdown annotations
Per maintainer review (#4379):
- Move the per-classification-level review frequencies / conditions out of the
  control description and into the annotation field, formatted as Markdown
  (bulleted list with the level names in bold).
- For 2-3-1-2, drop the redundant "applicable for Public and Confidential"
  wording since the implementation groups already convey applicability; keep
  only the BYOD-prohibited note for Secret and Top Secret.
- Add the official source link to the library description.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/excel/dcc/dcc-1-2022.xlsx
+++ b/tools/excel/dcc/dcc-1-2022.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NCA Data Cybersecurity Controls (DCC-1:2022), an extension of the Essential Cybersecurity Controls (ECC) focused on protecting data across its lifecycle. 3 main domains / 11 subdomains / 19 main controls / 47 subcontrols. Controls apply to four data classification levels (Public, Confidential, Secret, Top Secret), modelled here as implementation groups. Reference: https://nca.gov.sa</t>
+          <t>NCA Data Cybersecurity Controls (DCC-1:2022), an extension of the Essential Cybersecurity Controls (ECC) focused on protecting data across its lifecycle. 3 main domains / 11 subdomains / 19 main controls / 47 subcontrols. Controls apply to four data classification levels (Public, Confidential, Secret, Top Secret), modelled here as implementation groups. Source: https://cdn.nca.gov.sa/api/public/cms/files/1c2cfb9c-7788-4549-9f29-f337500f1787_Data-Cybersecurity-Controls-.pdf</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -840,7 +840,8 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="120" customWidth="1" min="6" max="6"/>
+    <col width="110" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -874,6 +875,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>annotation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr"/>
@@ -892,6 +898,7 @@
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr"/>
@@ -914,6 +921,7 @@
           <t>To ensure that cybersecurity controls are implemented and in compliance with organizational policies and procedures, as well as related national and international laws, regulations and agreements.</t>
         </is>
       </c>
+      <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -937,7 +945,12 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>With reference to ECC control 1-8-1, the cybersecurity function in the organization must review the implementation of the Data Cybersecurity Controls as specified for each data classification level. Review frequency: at least annually for all classification levels.</t>
+          <t>With reference to ECC control 1-8-1, the cybersecurity function in the organization must review the implementation of the Data Cybersecurity Controls as specified for each data classification level.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Review frequency: at least annually for all classification levels.</t>
         </is>
       </c>
     </row>
@@ -963,7 +976,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>With reference to ECC control 1-8-2, cybersecurity review and audit must be conducted periodically by independent parties outside the organization's cybersecurity function as specified for each data classification level. Review frequency: Public and Confidential at least every 2 years; Secret and Top Secret at least annually.</t>
+          <t>With reference to ECC control 1-8-2, cybersecurity review and audit must be conducted periodically by independent parties outside the organization's cybersecurity function as specified for each data classification level.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Review frequency:
+* **Public** and **Confidential** at least every 2 years
+* **Secret** and **Top Secret** at least annually</t>
         </is>
       </c>
     </row>
@@ -988,6 +1008,7 @@
           <t>To ensure that cybersecurity risks and requirements related to personnel (employees and contractors) are managed efficiently prior to employment, during employment and after termination/separation as per organizational policies and procedures, and related laws and regulations.</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -1006,6 +1027,7 @@
           <t>In addition to the subcontrols in the ECC control 1-9-3, cybersecurity requirements in human resources prior to employment, during employment and after termination/separation must include at least the following:</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1032,6 +1054,7 @@
           <t>Screening and vetting candidates in jobs related to data handling.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1058,6 +1081,7 @@
           <t>A signed agreement by personnel pledging to not use social media, communication applications or personal cloud storage to create, store or share the organization's data, with the exception of secure communication applications approved by relevant authorities.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr"/>
@@ -1080,6 +1104,7 @@
           <t>To ensure that personnel are aware of their cybersecurity responsibilities and have the required cybersecurity awareness. It is also to ensure that personnel are provided with the required cybersecurity training, skills and credentials needed to accomplish their cybersecurity responsibilities and to protect the organization's information and technology assets.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
@@ -1098,6 +1123,7 @@
           <t>In addition to the subcontrols in ECC control 1-10-3, the cybersecurity awareness program must cover topics related to data protection, including the following:</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1124,6 +1150,7 @@
           <t>Risks of data leakage and unauthorized access to data during its lifecycle.</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1150,6 +1177,7 @@
           <t>Secure handling of classified data while traveling and outside the workplace.</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1176,6 +1204,7 @@
           <t>Secure handling of data during meetings (virtual and in-person).</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1202,6 +1231,7 @@
           <t>Secure use of printers, scanners and copy machines.</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1228,6 +1258,7 @@
           <t>Procedures for secure data disposal.</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1254,6 +1285,7 @@
           <t>Risks of sharing documents and information through non-secure channels.</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1280,6 +1312,7 @@
           <t>Cybersecurity risks related to the use of external storage media.</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr"/>
@@ -1298,6 +1331,7 @@
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr"/>
@@ -1320,6 +1354,7 @@
           <t>To ensure the secure and restricted logical access to information and technology assets in order to prevent unauthorized access and allow only authorized access for users which are necessary to accomplish assigned tasks.</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -1338,6 +1373,7 @@
           <t>In addition to the subcontrols in ECC control 2-2-3, cybersecurity requirements for identity and access management must cover at least the following:</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1364,6 +1400,7 @@
           <t>Strict restriction to allow only the minimum number of personnel accessing, viewing and sharing data based on lists of privileges limited to Saudi national employees unless exempted by the Authorizing Official (the head of the organization or his/her delegate) and those lists are approved by the Authorizing Official.</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1390,6 +1427,7 @@
           <t>Prohibiting the sharing of approved lists of privileges with unauthorized persons.</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1416,6 +1454,7 @@
           <t>Managing identities and access rights to view data using Privileged Access Management systems.</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1439,7 +1478,14 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>In addition to ECC subcontrol 2-2-3-5, the approved lists of privileges and privileges used to handle data must be reviewed as specified for each data classification level. Review frequency: Public and Confidential at least annually; Secret and Top Secret at least every 3 months.</t>
+          <t>In addition to ECC subcontrol 2-2-3-5, the approved lists of privileges and privileges used to handle data must be reviewed as specified for each data classification level.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Review frequency:
+* **Public** and **Confidential** at least annually
+* **Secret** and **Top Secret** at least every 3 months</t>
         </is>
       </c>
     </row>
@@ -1464,6 +1510,7 @@
           <t>To ensure the protection of information systems and information processing facilities (including workstations and infrastructures) against cyber risks.</t>
         </is>
       </c>
+      <c r="G26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
@@ -1482,6 +1529,7 @@
           <t>In addition to the subcontrols in ECC control 2-3-3, cybersecurity requirements for Information System and Information Processing Facilities Protection must include at least the following:</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1505,7 +1553,14 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Applying security patches and updates from the time of announcement on systems used to handle data as specified for each data classification level. Frequency: Public and Confidential at least every month; Secret and Top Secret immediately.</t>
+          <t>Applying security patches and updates from the time of announcement on systems used to handle data as specified for each data classification level.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Frequency:
+* **Public** and **Confidential** at least every month
+* **Secret** and **Top Secret** immediately</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1586,14 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Reviewing the security configuration and hardening of systems used to handle data as specified for each data classification level. Frequency: Public and Confidential at least annually; Secret and Top Secret at least every 6 months.</t>
+          <t>Reviewing the security configuration and hardening of systems used to handle data as specified for each data classification level.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Frequency:
+* **Public** and **Confidential** at least annually
+* **Secret** and **Top Secret** at least every 6 months</t>
         </is>
       </c>
     </row>
@@ -1560,6 +1622,7 @@
           <t>Reviewing and hardening the default configuration (e.g., default passwords and backgrounds) of the technology assets used to handle the data.</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1586,6 +1649,7 @@
           <t>Disabling the Print Screen or Screen Capture features on the devices that create or process documents.</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr"/>
@@ -1608,6 +1672,7 @@
           <t>To ensure the protection of mobile devices (including laptops, smartphones, tablets) from cyber risks and to ensure the secure handling of the organization's information (including sensitive information) while utilizing Bring Your Own Device (BYOD) policy.</t>
         </is>
       </c>
+      <c r="G32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
@@ -1626,6 +1691,7 @@
           <t>In addition to the subcontrols in ECC control 2-6-3, cybersecurity requirements for mobile devices must cover at least the following:</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1652,6 +1718,7 @@
           <t>Centrally managing the organization's owned mobile devices using Mobile Device Management (MDM) system and activating the remote wipe feature.</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1675,7 +1742,12 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Centrally managing BYOD devices using Mobile Device Management (MDM) system and activating the remote wipe feature. Applicability by classification level: applicable for Public and Confidential; for Secret and Top Secret the use of BYOD devices is prohibited.</t>
+          <t>Centrally managing BYOD devices using Mobile Device Management (MDM) system and activating the remote wipe feature.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Applicability by classification level: for **Secret** and **Top Secret** the use of BYOD devices is prohibited.</t>
         </is>
       </c>
     </row>
@@ -1700,6 +1772,7 @@
           <t>To ensure the confidentiality, integrity and availability of organization's data and information as per organizational policies and procedures, and related laws and regulations.</t>
         </is>
       </c>
+      <c r="G36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
@@ -1718,6 +1791,7 @@
           <t>In addition to ECC control 2-7-3, cybersecurity requirements for data and information protection must cover at least the following:</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1744,6 +1818,7 @@
           <t>Using Watermark feature to label the whole document when creating, storing, printing, on the screen and on each copy so that the symbol can be traced to the user or device level.</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1770,6 +1845,7 @@
           <t>Using Data Leakage Prevention technologies and Rights Management technologies.</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1796,6 +1872,7 @@
           <t>Prohibiting the use of data in any environment other than the production environment, except after conducting a risk assessment and applying controls to protect that data, such as data masking or data scrambling techniques.</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1822,6 +1899,7 @@
           <t>Using brand protection service to protect the organization's identity from impersonation.</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr"/>
@@ -1844,6 +1922,7 @@
           <t>To ensure the proper and efficient use of cryptography to protect information assets as per organizational policies and procedures, and related laws and regulations.</t>
         </is>
       </c>
+      <c r="G42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
@@ -1862,6 +1941,7 @@
           <t>In addition to the subcontrols in ECC control 2-8-3, cybersecurity requirements for cryptography must cover at least the following:</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1888,6 +1968,7 @@
           <t>Using secure and up-to-date cryptographic methods and algorithms when creating, storing, transmitting data, and for overall network communication medium; as per the requirements of the "advanced level" in the National Cryptographic Standards (NCS-1:2020).</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1914,6 +1995,7 @@
           <t>Using secure and up-to-date cryptographic methods and algorithms when creating, storing, transmitting data, and for overall network communication medium; as per the requirements of the "moderate level" in the National Cryptographic Standards (NCS-1:2020).</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr"/>
@@ -1936,6 +2018,7 @@
           <t>To ensure a secure data disposal as per organizational policies and procedures, and related laws and regulations.</t>
         </is>
       </c>
+      <c r="G46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
@@ -1954,6 +2037,7 @@
           <t>Cybersecurity requirements for secure data disposal must cover at least the following:</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1980,6 +2064,7 @@
           <t>Identification of technologies, tools and procedures for the implementation of secure data disposal according to the data classification level.</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2006,6 +2091,7 @@
           <t>When storage media is no longer needed, it must be securely disposed by using the technologies, tools and procedures identified in subcontrol 2-6-1-1.</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2032,6 +2118,7 @@
           <t>When storage media needs to be re-used, data must be securely erased (secure erasure) in a manner it cannot be recovered.</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2058,6 +2145,7 @@
           <t>Implementation of secure data disposal or erasure operations referred to in sub-controls 2-6-1-2 and 2-6-1-3 must be verified.</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2084,6 +2172,7 @@
           <t>Keeping a record of all secure data disposal and erasure operations that have been conducted.</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2107,7 +2196,14 @@
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>The implementation of the secure data disposal requirements must be reviewed as specified for each data classification level. Review frequency: Public and Confidential at least annually; Secret and Top Secret at least every 6 months.</t>
+          <t>The implementation of the secure data disposal requirements must be reviewed as specified for each data classification level.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Review frequency:
+* **Public** and **Confidential** at least annually
+* **Secret** and **Top Secret** at least every 6 months</t>
         </is>
       </c>
     </row>
@@ -2132,6 +2228,7 @@
           <t>To ensure secure handling of data when using Printers, Scanners and Copy Machines.</t>
         </is>
       </c>
+      <c r="G54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2158,6 +2255,7 @@
           <t>Cybersecurity requirements for protecting printers, scanners and copy machines must be defined, documented and approved.</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2184,6 +2282,7 @@
           <t>Cybersecurity requirements for printers, scanners and copy machines must be implemented.</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
@@ -2202,6 +2301,7 @@
           <t>Cybersecurity requirements for printers, scanners and copy machines must cover at least the following:</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2228,6 +2328,7 @@
           <t>Disabling the temporary storage feature.</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2254,6 +2355,7 @@
           <t>Enabling authentication on centralized printers, scanners and copy machines and requiring it before usage.</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2280,6 +2382,7 @@
           <t>Securely retaining (for a period not less than 12 months) logs of printers, scanners and copy machines usage.</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2306,6 +2409,7 @@
           <t>Enabling and protecting CCTV logs which are used to monitor centralized printers, scanners and copy machines areas.</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2332,6 +2436,7 @@
           <t>Using cross-shredding devices, to securely dispose documents when no longer needed.</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2355,7 +2460,14 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Implementation of cybersecurity requirements for printers, scanners and copy machines must be reviewed as specified for each data classification level. Review frequency: Public and Confidential at least every 3 years; Secret and Top Secret at least annually.</t>
+          <t>Implementation of cybersecurity requirements for printers, scanners and copy machines must be reviewed as specified for each data classification level.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Review frequency:
+* **Public** and **Confidential** at least every 3 years
+* **Secret** and **Top Secret** at least annually</t>
         </is>
       </c>
     </row>
@@ -2376,6 +2488,7 @@
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr"/>
+      <c r="G64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr"/>
@@ -2398,6 +2511,7 @@
           <t>To ensure the protection of assets against the cybersecurity risks related to third parties including outsourcing, managed services, and consultancy services as per organizational policies and procedures, and related laws and regulations.</t>
         </is>
       </c>
+      <c r="G65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
@@ -2416,6 +2530,7 @@
           <t>In addition to the controls in ECC subdomain 4-1, cybersecurity requirements for third-parties cybersecurity must include at least the following:</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2442,6 +2557,7 @@
           <t>Screening or vetting third-party employees who have access to the data.</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2468,6 +2584,7 @@
           <t>Requiring contractual commitment by third-parties to securely dispose the organization's data at the end of the contract or in case of contract termination, including providing evidences of such disposal to the organization.</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2494,6 +2611,7 @@
           <t>Documenting all data sharing operations within third-parties, including data sharing justification.</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2520,6 +2638,7 @@
           <t>When transferring data outside the kingdom, the capability of the hosting organization abroad to safeguard data must be verified, approval of the Authorizing Official must be obtained and complying with related laws and regulations.</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2546,6 +2665,7 @@
           <t>Requiring third-parties to notify the organization immediately in case of cybersecurity incident that may affect data being shared or created.</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2572,6 +2692,7 @@
           <t>Reclassifying data to the least level to achieve the objective before sharing it with third-parties using data masking or data scrambling techniques.</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr"/>
@@ -2590,6 +2711,7 @@
           <t>In alignment with related laws and regulations, and in addition to the applicable controls in ECC and controls within DCC domains (1), (2), and (3), cybersecurity requirements when dealing with consultancy services that work on high-sensitivity strategic projects at the national level must cover at least the following:</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2616,6 +2738,7 @@
           <t>Screening or vetting consultancy services employees who have access to the data.</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2642,6 +2765,7 @@
           <t>Requiring contractual commitment by consultancy services including employees non-disclosure agreements and secure disposal the organization's data at the end of the contract or in case of contract termination, including providing evidences of such disposal to the organization.</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2668,6 +2792,7 @@
           <t>Documenting all data sharing operations within consultancy services, including data sharing justification.</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2694,6 +2819,7 @@
           <t>Requiring consultancy services to notify the organization immediately in case of cybersecurity incident that may affect data that has been shared or created.</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2720,6 +2846,7 @@
           <t>Reclassifying data to the least level to achieve the objective before sharing it with consultancy services using data masking or data scrambling techniques.</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2746,6 +2873,7 @@
           <t>Dedicating a closed room for the consultancy services employees to perform their work, in addition to providing dedicated organization owned devices to share and process data.</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2772,6 +2900,7 @@
           <t>Activating access control system to allow only authorized access to the closed room.</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2798,6 +2927,7 @@
           <t>Preventing carrying out of devices, storage media and documents outside the closed room, as well as the entry of any other electronic devices.</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>